<commit_message>
novas implementações, executável local
</commit_message>
<xml_diff>
--- a/visitas_gre_ficticias.xlsx
+++ b/visitas_gre_ficticias.xlsx
@@ -1,20 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29512"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1FFF18EA-4462-4435-8834-4ACC28AEC609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="108">
   <si>
     <t>Escola</t>
   </si>
@@ -40,298 +57,310 @@
     <t>Escola de Referência em Ensino Fundamental e Médio Caio Pereira</t>
   </si>
   <si>
+    <t>15/03/2025</t>
+  </si>
+  <si>
+    <t>Ana Lima (GRE Mata Sul)</t>
+  </si>
+  <si>
+    <t>Maria Silva</t>
+  </si>
+  <si>
+    <t>Problema no laboratório de informática</t>
+  </si>
+  <si>
+    <t>Verificar computadores</t>
+  </si>
+  <si>
+    <t>5 computadores não ligam.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Fundamental e Médio Dona Maria Teresa</t>
   </si>
   <si>
+    <t>18/03/2025</t>
+  </si>
+  <si>
+    <t>Bruno Costa (GRE Recife Norte)</t>
+  </si>
+  <si>
+    <t>João Pereira</t>
+  </si>
+  <si>
+    <t>Formação SAEPE para professores</t>
+  </si>
+  <si>
+    <t>Agendar formação</t>
+  </si>
+  <si>
+    <t>Professores com dúvidas sobre a plataforma.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Fundamental e Médio Gilberto Freyre</t>
   </si>
   <si>
+    <t>02/04/2025</t>
+  </si>
+  <si>
+    <t>Carlos Souza</t>
+  </si>
+  <si>
+    <t>Acompanhamento pedagógico 9º ano</t>
+  </si>
+  <si>
+    <t>Reunião com coordenação</t>
+  </si>
+  <si>
+    <t>Alunos com baixa frequência.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Fundamental e Médio Gov Barbosa Lima</t>
   </si>
   <si>
+    <t>05/04/2025</t>
+  </si>
+  <si>
+    <t>Mariana Dias (GRE Agreste)</t>
+  </si>
+  <si>
+    <t>Rita de Cássia</t>
+  </si>
+  <si>
+    <t>Internet lenta na biblioteca</t>
+  </si>
+  <si>
+    <t>Abrir chamado técnico</t>
+  </si>
+  <si>
+    <t>Sinal de Wi-Fi fraco.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Fundamental e Médio Jarbas Pernambuco</t>
   </si>
   <si>
+    <t>10/04/2025</t>
+  </si>
+  <si>
+    <t>Pedro Almeida</t>
+  </si>
+  <si>
+    <t>Solicitação de mais livros didáticos</t>
+  </si>
+  <si>
+    <t>Enviar para a secretaria</t>
+  </si>
+  <si>
+    <t>Faltam livros de Matemática.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Fundamental e Médio Liceu de Artes e Ofícios</t>
   </si>
   <si>
+    <t>12/04/2025</t>
+  </si>
+  <si>
+    <t>Lúcia Ferreira</t>
+  </si>
+  <si>
+    <t>Verificação estrutural - telhado</t>
+  </si>
+  <si>
+    <t>Relatório para engenharia</t>
+  </si>
+  <si>
+    <t>Infiltração na sala 10.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Médio de Beberibe</t>
   </si>
   <si>
+    <t>15/04/2025</t>
+  </si>
+  <si>
+    <t>Sônia Braga</t>
+  </si>
+  <si>
+    <t>Problema no quadro elétrico</t>
+  </si>
+  <si>
+    <t>Chamar eletricista</t>
+  </si>
+  <si>
+    <t>Quedas de energia constantes.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Médio de Camaragibe</t>
   </si>
   <si>
+    <t>20/04/2025</t>
+  </si>
+  <si>
+    <t>Marcos Andrade</t>
+  </si>
+  <si>
+    <t>Formação sobre novo currículo</t>
+  </si>
+  <si>
+    <t>Disponibilizar material</t>
+  </si>
+  <si>
+    <t>Equipe pedagógica alinhada.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Médio de Igarassu</t>
   </si>
   <si>
+    <t>02/05/2025</t>
+  </si>
+  <si>
+    <t>Planejamento de aulas de reforço</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Visita de rotina.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Médio de Olinda</t>
   </si>
   <si>
+    <t>05/05/2025</t>
+  </si>
+  <si>
+    <t>Tânia Guedes</t>
+  </si>
+  <si>
+    <t>Auditoria da merenda escolar</t>
+  </si>
+  <si>
+    <t>Relatório enviado</t>
+  </si>
+  <si>
+    <t>Tudo em conformidade.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Médio de Paulista</t>
   </si>
   <si>
+    <t>10/05/2025</t>
+  </si>
+  <si>
+    <t>José Carlos</t>
+  </si>
+  <si>
+    <t>Entrega de materiais esportivos</t>
+  </si>
+  <si>
+    <t>Recebido pela coordenação</t>
+  </si>
+  <si>
+    <t>Faltaram 2 bolas de vôlei.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Médio de São Lourenço da Mata</t>
   </si>
   <si>
+    <t>12/05/2025</t>
+  </si>
+  <si>
+    <t>Vera Lins</t>
+  </si>
+  <si>
+    <t>Problema no ar condicionado da diretoria</t>
+  </si>
+  <si>
+    <t>Manutenção agendada</t>
+  </si>
+  <si>
+    <t>Filtro precisa ser trocado.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Médio Ginásio Pernambucano</t>
   </si>
   <si>
+    <t>15/05/2025</t>
+  </si>
+  <si>
+    <t>Fábio Borges</t>
+  </si>
+  <si>
+    <t>Acompanhamento de projetos</t>
+  </si>
+  <si>
+    <t>Projetos de ciências em andamento.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Médio Gov. Eraldo Gueiros</t>
   </si>
   <si>
+    <t>20/05/2025</t>
+  </si>
+  <si>
+    <t>Sandra Melo</t>
+  </si>
+  <si>
+    <t>Verificação de transporte escolar</t>
+  </si>
+  <si>
+    <t>Ajustar rotas</t>
+  </si>
+  <si>
+    <t>Alguns alunos estão chegando atrasados.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Médio Nóbrega</t>
   </si>
   <si>
+    <t>22/05/2025</t>
+  </si>
+  <si>
+    <t>Cláudia Leite</t>
+  </si>
+  <si>
+    <t>Reunião sobre evasão escolar</t>
+  </si>
+  <si>
+    <t>Criar comitê de pais</t>
+  </si>
+  <si>
+    <t>A evasão aumentou 5% no último bimestre.</t>
+  </si>
+  <si>
     <t>Escola de Referência em Ensino Médio Oliveira Lima</t>
   </si>
   <si>
-    <t>15/03/2025</t>
-  </si>
-  <si>
-    <t>18/03/2025</t>
-  </si>
-  <si>
-    <t>02/04/2025</t>
-  </si>
-  <si>
-    <t>05/04/2025</t>
-  </si>
-  <si>
-    <t>10/04/2025</t>
-  </si>
-  <si>
-    <t>12/04/2025</t>
-  </si>
-  <si>
-    <t>15/04/2025</t>
-  </si>
-  <si>
-    <t>20/04/2025</t>
-  </si>
-  <si>
-    <t>02/05/2025</t>
-  </si>
-  <si>
-    <t>05/05/2025</t>
-  </si>
-  <si>
-    <t>10/05/2025</t>
-  </si>
-  <si>
-    <t>12/05/2025</t>
-  </si>
-  <si>
-    <t>15/05/2025</t>
-  </si>
-  <si>
-    <t>20/05/2025</t>
-  </si>
-  <si>
-    <t>22/05/2025</t>
-  </si>
-  <si>
     <t>25/05/2025</t>
   </si>
   <si>
-    <t>Ana Lima (GRE Mata Sul)</t>
-  </si>
-  <si>
-    <t>Bruno Costa (GRE Recife Norte)</t>
-  </si>
-  <si>
-    <t>Mariana Dias (GRE Agreste)</t>
-  </si>
-  <si>
-    <t>Maria Silva</t>
-  </si>
-  <si>
-    <t>João Pereira</t>
-  </si>
-  <si>
-    <t>Carlos Souza</t>
-  </si>
-  <si>
-    <t>Rita de Cássia</t>
-  </si>
-  <si>
-    <t>Pedro Almeida</t>
-  </si>
-  <si>
-    <t>Lúcia Ferreira</t>
-  </si>
-  <si>
-    <t>Sônia Braga</t>
-  </si>
-  <si>
-    <t>Marcos Andrade</t>
-  </si>
-  <si>
-    <t>Tânia Guedes</t>
-  </si>
-  <si>
-    <t>José Carlos</t>
-  </si>
-  <si>
-    <t>Vera Lins</t>
-  </si>
-  <si>
-    <t>Fábio Borges</t>
-  </si>
-  <si>
-    <t>Sandra Melo</t>
-  </si>
-  <si>
-    <t>Cláudia Leite</t>
-  </si>
-  <si>
     <t>Ricardo Nunes</t>
   </si>
   <si>
-    <t>Problema no laboratório de informática</t>
-  </si>
-  <si>
-    <t>Formação SAEPE para professores</t>
-  </si>
-  <si>
-    <t>Acompanhamento pedagógico 9º ano</t>
-  </si>
-  <si>
-    <t>Internet lenta na biblioteca</t>
-  </si>
-  <si>
-    <t>Solicitação de mais livros didáticos</t>
-  </si>
-  <si>
-    <t>Verificação estrutural - telhado</t>
-  </si>
-  <si>
-    <t>Problema no quadro elétrico</t>
-  </si>
-  <si>
-    <t>Formação sobre novo currículo</t>
-  </si>
-  <si>
-    <t>Planejamento de aulas de reforço</t>
-  </si>
-  <si>
-    <t>Auditoria da merenda escolar</t>
-  </si>
-  <si>
-    <t>Entrega de materiais esportivos</t>
-  </si>
-  <si>
-    <t>Problema no ar condicionado da diretoria</t>
-  </si>
-  <si>
-    <t>Acompanhamento de projetos</t>
-  </si>
-  <si>
-    <t>Verificação de transporte escolar</t>
-  </si>
-  <si>
-    <t>Reunião sobre evasão escolar</t>
-  </si>
-  <si>
     <t>Inspeção de bebedouros</t>
   </si>
   <si>
-    <t>Verificar computadores</t>
-  </si>
-  <si>
-    <t>Agendar formação</t>
-  </si>
-  <si>
-    <t>Reunião com coordenação</t>
-  </si>
-  <si>
-    <t>Abrir chamado técnico</t>
-  </si>
-  <si>
-    <t>Enviar para a secretaria</t>
-  </si>
-  <si>
-    <t>Relatório para engenharia</t>
-  </si>
-  <si>
-    <t>Chamar eletricista</t>
-  </si>
-  <si>
-    <t>Disponibilizar material</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Relatório enviado</t>
-  </si>
-  <si>
-    <t>Recebido pela coordenação</t>
-  </si>
-  <si>
-    <t>Manutenção agendada</t>
-  </si>
-  <si>
-    <t>Ajustar rotas</t>
-  </si>
-  <si>
-    <t>Criar comitê de pais</t>
-  </si>
-  <si>
     <t>Trocar filtros</t>
   </si>
   <si>
-    <t>5 computadores não ligam.</t>
-  </si>
-  <si>
-    <t>Professores com dúvidas sobre a plataforma.</t>
-  </si>
-  <si>
-    <t>Alunos com baixa frequência.</t>
-  </si>
-  <si>
-    <t>Sinal de Wi-Fi fraco.</t>
-  </si>
-  <si>
-    <t>Faltam livros de Matemática.</t>
-  </si>
-  <si>
-    <t>Infiltração na sala 10.</t>
-  </si>
-  <si>
-    <t>Quedas de energia constantes.</t>
-  </si>
-  <si>
-    <t>Equipe pedagógica alinhada.</t>
-  </si>
-  <si>
-    <t>Visita de rotina.</t>
-  </si>
-  <si>
-    <t>Tudo em conformidade.</t>
-  </si>
-  <si>
-    <t>Faltaram 2 bolas de vôlei.</t>
-  </si>
-  <si>
-    <t>Filtro precisa ser trocado.</t>
-  </si>
-  <si>
-    <t>Projetos de ciências em andamento.</t>
-  </si>
-  <si>
-    <t>Alguns alunos estão chegando atrasados.</t>
-  </si>
-  <si>
-    <t>A evasão aumentou 5% no último bimestre.</t>
-  </si>
-  <si>
     <t>Bebedouro do pátio com vazamento.</t>
+  </si>
+  <si>
+    <t>Escola de Teste</t>
+  </si>
+  <si>
+    <t>Cláudio</t>
+  </si>
+  <si>
+    <t>Teste</t>
+  </si>
+  <si>
+    <t>teste</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -384,10 +413,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -395,13 +427,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -439,7 +479,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -473,6 +513,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -507,9 +548,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -682,9 +724,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="96.28515625" customWidth="1"/>
+    <col min="2" max="2" width="64.28515625" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="4" max="4" width="47.42578125" customWidth="1"/>
+    <col min="6" max="6" width="40.28515625" customWidth="1"/>
+    <col min="7" max="7" width="51" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
@@ -714,367 +764,390 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>88</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>74</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>89</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
         <v>25</v>
       </c>
-      <c r="C4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E4" t="s">
-        <v>59</v>
-      </c>
-      <c r="F4" t="s">
-        <v>75</v>
-      </c>
       <c r="G4" t="s">
-        <v>90</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>32</v>
       </c>
       <c r="G5" t="s">
-        <v>91</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="G6" t="s">
-        <v>92</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E7" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
+        <v>44</v>
       </c>
       <c r="G7" t="s">
-        <v>93</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="D8" t="s">
         <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F8" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>56</v>
       </c>
       <c r="G9" t="s">
-        <v>95</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="G10" t="s">
-        <v>96</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" t="s">
         <v>16</v>
       </c>
-      <c r="B11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
-      </c>
       <c r="D11" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="E11" t="s">
         <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="G11" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="F12" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="G12" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>77</v>
       </c>
       <c r="E13" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F13" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="G13" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
+        <v>82</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>83</v>
       </c>
       <c r="E14" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="G14" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>87</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="E15" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="G15" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>92</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>93</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>94</v>
       </c>
       <c r="E16" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="F16" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="G16" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>98</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>99</v>
       </c>
       <c r="C17" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>56</v>
+        <v>100</v>
       </c>
       <c r="E17" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="F17" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="G17" t="s">
         <v>103</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" s="2">
+        <v>46017</v>
+      </c>
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" t="s">
+        <v>105</v>
+      </c>
+      <c r="E18" t="s">
+        <v>106</v>
+      </c>
+      <c r="F18" t="s">
+        <v>106</v>
+      </c>
+      <c r="G18" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>